<commit_message>
Generated Assessment for FinOps Foundation
</commit_message>
<xml_diff>
--- a/assessments/FinOps Foundation/assessment.xlsx
+++ b/assessments/FinOps Foundation/assessment.xlsx
@@ -17,7 +17,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1232" uniqueCount="427">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1237" uniqueCount="436">
   <si>
     <t>Sum of Weights</t>
   </si>
@@ -995,6 +995,12 @@
   </si>
   <si>
     <t>2.1.0</t>
+  </si>
+  <si>
+    <t>2.0.0</t>
+  </si>
+  <si>
+    <t>1.9.0</t>
   </si>
   <si>
     <t>1.6.1</t>
@@ -1159,6 +1165,21 @@
 10*Ceil(x/5)</t>
   </si>
   <si>
+    <t>* Implement architecture changes in time boxed iterations rather than big migrations
+* Track actual cost outcomes vs estimated savings documented in prior trade off analysis
+* Define and monitor success metrics (cost delta, performance, reliability) for each iteration
+* Hold structured retrospectives after each iteration to capture lessons learned
+* Feed iteration outcomes back into the modernization backlog to reprioritize remaining work
+10*Ceil(x/5)</t>
+  </si>
+  <si>
+    <t>* Document and publish cost savings and performance outcomes achieved through architecture changes
+* Update internal architecture reference guides and design patterns with validated approaches
+* Share case studies and reusable blueprints with engineering teams to accelerate adoption
+* Establish a regular cadence to refresh published benefits data and retire outdated references
+10*Ceil(x/4)</t>
+  </si>
+  <si>
     <t>* Process defined for new accounts and resources deployed
 * Train teams on process
 * Automate process
@@ -1173,10 +1194,10 @@
 10*Ceil(x/5)</t>
   </si>
   <si>
-    <t>* Data based on existing patterns
-* Proactive investigations and interviews with teams
-* Proactive self reporting by the business and/or teams
-* 100% catch rate of spikes before they happen
+    <t>* Collect data based on existing patterns observed in spend
+* Conduct proactive investigations and interviews with teams
+* Gather existing self reporting by the business and/or teams
+* Factor in expected increases to the forecast model
 10*Ceil(x/4)</t>
   </si>
   <si>
@@ -1320,6 +1341,32 @@
 * RCA completed after alerts
 10*Ceil(x/6)
 </t>
+  </si>
+  <si>
+    <t>Denominator: all anomalies detected during the review period. A field item is met when the field is
+populated on 90% or more of those records.
+* Single system of record
+* Scope fields populated (billing account, service, region, and a named accountable owner)
+* Impact fields populated (variance amount in the reporting currency, and the start and end of the
+  period the variance covers)
+* Timeline fields populated (first occurrence, detection, notification, and resolution timestamps)
+* Disposition field populated (true, expected change, or false)
+* Retention and queryability (records retained for at least 13 months and queryable by scope,
+  disposition, and root cause)
+10*Ceil(x/6)</t>
+  </si>
+  <si>
+    <t>Denominator: anomalies recorded with a true positive disposition during the review period. Items 1
+through 4 are met when the stated field is populated on 90% or more of those records.
+1. Owner and due date (each record carries a named accountable owner and an analysis due date)
+2. Root cause recorded (each record carries a root cause entry naming the change that triggered it)
+3. Cause classified (each root cause assigned exactly one category from a published, fixed
+   category list)
+4. Remediation recorded (each record carries a remediation action, its completion date, and the
+   measured spend delta over the period following the fix)
+5. Preventive control registered (every cause category observed 3 or more times in the trailing
+   12 months has a linked policy, guardrail, budget, or detection rule)
+10*Ceil(x/5)</t>
   </si>
   <si>
     <t>* Number of detections per time period
@@ -1333,6 +1380,25 @@
 10*Ceil(x/8)</t>
   </si>
   <si>
+    <t>* Weighted sum
+  Alert precision (score x4),
+  Missed anomalies (score x3),
+  Tuning cadence (score x2),
+  Tuning governance (score x1).
+  Max raw (50)
+* Alert_Precision: Alerts confirmed as true positives divided by all alerts raised in the review period
+  (0=Not measured, 1&lt;50%, 2=50-69%, 3=70-84%, 4=85-94%, 5=95%+)
+* Missed_Anomalies: Share of anomalies first found by invoice review, budget variance, or an owner
+  (0=Not measured, 1&gt;25%, 2=10-25%, 3=5-9%, 4=1-4%, 5&lt;1%)
+* Tuning_Cadence: How often thresholds are reviewed and adjusted against observed outcomes
+  (0=Never, 1=Ad-hoc, 2=Annual, 3=Quarterly, 4=Monthly, 5=Continuous or automated)
+* Tuning_Governance: How a threshold change is decided and recorded
+  (0=Undocumented, 1=Changed by one person, 2=Documented with rationale,
+  3=Reviewed with the alert recipients, 4=Version controlled and auditable,
+  5=Version controlled and replayed against historical anomalies before release)
+* Output Range (0-50)</t>
+  </si>
+  <si>
     <t xml:space="preserve">* Define data quality (complete, valid, etc.)
 * Manual quality checks
 * Automated checks (null % on required fields/tags)
@@ -1459,6 +1525,9 @@
     <t>[{'Score': 0, 'Condition': 'No items completed'}, {'Score': 2, 'Condition': '1 item completed'}, {'Score': 3, 'Condition': '2 items completed'}, {'Score': 4, 'Condition': '3 items completed'}, {'Score': 5, 'Condition': '4 items completed'}, {'Score': 7, 'Condition': '5 items completed'}, {'Score': 8, 'Condition': '6 items completed'}, {'Score': 9, 'Condition': '7 items completed'}, {'Score': 10, 'Condition': '8 items completed'}]</t>
   </si>
   <si>
+    <t>[{'Score': 0, 'Condition': 'Low Maturity, Score Range (0-14)'}, {'Score': 4, 'Condition': 'Developing, Score Range (15-30)'}, {'Score': 7, 'Condition': 'Established, Score Range (31-42)'}, {'Score': 10, 'Condition': 'Optimizing, Score Range (43-50)'}]</t>
+  </si>
+  <si>
     <t>[{'Score': 0, 'Condition': 'Never'}, {'Score': 1, 'Condition': 'Monthly or greater'}, {'Score': 2, 'Condition': 'More than a week'}, {'Score': 3, 'Condition': '7 days'}, {'Score': 4, 'Condition': '5 days'}, {'Score': 6, 'Condition': '2 days'}, {'Score': 8, 'Condition': '1 day'}, {'Score': 10, 'Condition': 'Instant'}]</t>
   </si>
   <si>
@@ -1514,6 +1583,9 @@
   </si>
   <si>
     <t>0: No alerting to any owners</t>
+  </si>
+  <si>
+    <t>0: Low Maturity. Score Range (0-14)</t>
   </si>
   <si>
     <t>0: Never</t>
@@ -2867,7 +2939,7 @@
         <v>1</v>
       </c>
       <c r="H2" s="1" t="s">
-        <v>409</v>
+        <v>417</v>
       </c>
       <c r="I2">
         <f>F2*VALUE(LEFT(H2, FIND(":", H2)-1))</f>
@@ -2896,7 +2968,7 @@
         <v>1</v>
       </c>
       <c r="H3" s="1" t="s">
-        <v>409</v>
+        <v>417</v>
       </c>
       <c r="I3">
         <f>F3*VALUE(LEFT(H3, FIND(":", H3)-1))</f>
@@ -2925,7 +2997,7 @@
         <v>1</v>
       </c>
       <c r="H4" s="1" t="s">
-        <v>409</v>
+        <v>417</v>
       </c>
       <c r="I4">
         <f>F4*VALUE(LEFT(H4, FIND(":", H4)-1))</f>
@@ -2954,7 +3026,7 @@
         <v>1</v>
       </c>
       <c r="H5" s="1" t="s">
-        <v>410</v>
+        <v>418</v>
       </c>
       <c r="I5">
         <f>F5*VALUE(LEFT(H5, FIND(":", H5)-1))</f>
@@ -2983,7 +3055,7 @@
         <v>1</v>
       </c>
       <c r="H6" s="1" t="s">
-        <v>409</v>
+        <v>417</v>
       </c>
       <c r="I6">
         <f>F6*VALUE(LEFT(H6, FIND(":", H6)-1))</f>
@@ -3014,10 +3086,10 @@
         <v>1</v>
       </c>
       <c r="G7" s="1" t="s">
-        <v>327</v>
+        <v>329</v>
       </c>
       <c r="H7" s="1" t="s">
-        <v>411</v>
+        <v>419</v>
       </c>
       <c r="I7">
         <f>F7*VALUE(LEFT(H7, FIND(":", H7)-1))</f>
@@ -3046,10 +3118,10 @@
         <v>1</v>
       </c>
       <c r="G8" s="1" t="s">
-        <v>328</v>
+        <v>330</v>
       </c>
       <c r="H8" s="1" t="s">
-        <v>412</v>
+        <v>420</v>
       </c>
       <c r="I8">
         <f>F8*VALUE(LEFT(H8, FIND(":", H8)-1))</f>
@@ -3078,10 +3150,10 @@
         <v>1</v>
       </c>
       <c r="G9" s="1" t="s">
-        <v>329</v>
+        <v>331</v>
       </c>
       <c r="H9" s="1" t="s">
-        <v>412</v>
+        <v>420</v>
       </c>
       <c r="I9">
         <f>F9*VALUE(LEFT(H9, FIND(":", H9)-1))</f>
@@ -3110,10 +3182,10 @@
         <v>1</v>
       </c>
       <c r="G10" s="1" t="s">
-        <v>330</v>
+        <v>332</v>
       </c>
       <c r="H10" s="1" t="s">
-        <v>412</v>
+        <v>420</v>
       </c>
       <c r="I10">
         <f>F10*VALUE(LEFT(H10, FIND(":", H10)-1))</f>
@@ -3142,10 +3214,10 @@
         <v>1</v>
       </c>
       <c r="G11" s="1" t="s">
-        <v>331</v>
+        <v>333</v>
       </c>
       <c r="H11" s="1" t="s">
-        <v>412</v>
+        <v>420</v>
       </c>
       <c r="I11">
         <f>F11*VALUE(LEFT(H11, FIND(":", H11)-1))</f>
@@ -3176,7 +3248,7 @@
         <v>1</v>
       </c>
       <c r="H12" s="1" t="s">
-        <v>409</v>
+        <v>417</v>
       </c>
       <c r="I12">
         <f>F12*VALUE(LEFT(H12, FIND(":", H12)-1))</f>
@@ -3205,7 +3277,7 @@
         <v>1</v>
       </c>
       <c r="H13" s="1" t="s">
-        <v>409</v>
+        <v>417</v>
       </c>
       <c r="I13">
         <f>F13*VALUE(LEFT(H13, FIND(":", H13)-1))</f>
@@ -3234,7 +3306,7 @@
         <v>1</v>
       </c>
       <c r="H14" s="1" t="s">
-        <v>409</v>
+        <v>417</v>
       </c>
       <c r="I14">
         <f>F14*VALUE(LEFT(H14, FIND(":", H14)-1))</f>
@@ -3263,10 +3335,10 @@
         <v>1</v>
       </c>
       <c r="G15" s="1" t="s">
-        <v>332</v>
+        <v>334</v>
       </c>
       <c r="H15" s="1" t="s">
-        <v>412</v>
+        <v>420</v>
       </c>
       <c r="I15">
         <f>F15*VALUE(LEFT(H15, FIND(":", H15)-1))</f>
@@ -3295,7 +3367,7 @@
         <v>1</v>
       </c>
       <c r="H16" s="1" t="s">
-        <v>409</v>
+        <v>417</v>
       </c>
       <c r="I16">
         <f>F16*VALUE(LEFT(H16, FIND(":", H16)-1))</f>
@@ -3326,7 +3398,7 @@
         <v>1</v>
       </c>
       <c r="H17" s="1" t="s">
-        <v>409</v>
+        <v>417</v>
       </c>
       <c r="I17">
         <f>F17*VALUE(LEFT(H17, FIND(":", H17)-1))</f>
@@ -3355,7 +3427,7 @@
         <v>1</v>
       </c>
       <c r="H18" s="1" t="s">
-        <v>409</v>
+        <v>417</v>
       </c>
       <c r="I18">
         <f>F18*VALUE(LEFT(H18, FIND(":", H18)-1))</f>
@@ -3384,7 +3456,7 @@
         <v>1</v>
       </c>
       <c r="H19" s="1" t="s">
-        <v>409</v>
+        <v>417</v>
       </c>
       <c r="I19">
         <f>F19*VALUE(LEFT(H19, FIND(":", H19)-1))</f>
@@ -3413,7 +3485,7 @@
         <v>1</v>
       </c>
       <c r="H20" s="1" t="s">
-        <v>409</v>
+        <v>417</v>
       </c>
       <c r="I20">
         <f>F20*VALUE(LEFT(H20, FIND(":", H20)-1))</f>
@@ -3442,7 +3514,7 @@
         <v>1</v>
       </c>
       <c r="H21" s="1" t="s">
-        <v>409</v>
+        <v>417</v>
       </c>
       <c r="I21">
         <f>F21*VALUE(LEFT(H21, FIND(":", H21)-1))</f>
@@ -3471,7 +3543,7 @@
         <v>1</v>
       </c>
       <c r="H22" s="1" t="s">
-        <v>409</v>
+        <v>417</v>
       </c>
       <c r="I22">
         <f>F22*VALUE(LEFT(H22, FIND(":", H22)-1))</f>
@@ -3502,10 +3574,10 @@
         <v>1</v>
       </c>
       <c r="G23" s="1" t="s">
-        <v>333</v>
+        <v>335</v>
       </c>
       <c r="H23" s="1" t="s">
-        <v>413</v>
+        <v>421</v>
       </c>
       <c r="I23">
         <f>F23*VALUE(LEFT(H23, FIND(":", H23)-1))</f>
@@ -3534,10 +3606,10 @@
         <v>1</v>
       </c>
       <c r="G24" s="1" t="s">
-        <v>334</v>
+        <v>336</v>
       </c>
       <c r="H24" s="1" t="s">
-        <v>414</v>
+        <v>422</v>
       </c>
       <c r="I24">
         <f>F24*VALUE(LEFT(H24, FIND(":", H24)-1))</f>
@@ -3566,10 +3638,10 @@
         <v>1</v>
       </c>
       <c r="G25" s="1" t="s">
-        <v>335</v>
+        <v>337</v>
       </c>
       <c r="H25" s="1" t="s">
-        <v>415</v>
+        <v>423</v>
       </c>
       <c r="I25">
         <f>F25*VALUE(LEFT(H25, FIND(":", H25)-1))</f>
@@ -3598,10 +3670,10 @@
         <v>1</v>
       </c>
       <c r="G26" s="1" t="s">
-        <v>336</v>
+        <v>338</v>
       </c>
       <c r="H26" s="1" t="s">
-        <v>412</v>
+        <v>420</v>
       </c>
       <c r="I26">
         <f>F26*VALUE(LEFT(H26, FIND(":", H26)-1))</f>
@@ -3630,7 +3702,7 @@
         <v>1</v>
       </c>
       <c r="H27" s="1" t="s">
-        <v>409</v>
+        <v>417</v>
       </c>
       <c r="I27">
         <f>F27*VALUE(LEFT(H27, FIND(":", H27)-1))</f>
@@ -3661,10 +3733,10 @@
         <v>1</v>
       </c>
       <c r="G28" s="1" t="s">
-        <v>337</v>
+        <v>339</v>
       </c>
       <c r="H28" s="1" t="s">
-        <v>412</v>
+        <v>420</v>
       </c>
       <c r="I28">
         <f>F28*VALUE(LEFT(H28, FIND(":", H28)-1))</f>
@@ -3693,10 +3765,10 @@
         <v>1</v>
       </c>
       <c r="G29" s="1" t="s">
-        <v>338</v>
+        <v>340</v>
       </c>
       <c r="H29" s="1" t="s">
-        <v>412</v>
+        <v>420</v>
       </c>
       <c r="I29">
         <f>F29*VALUE(LEFT(H29, FIND(":", H29)-1))</f>
@@ -3725,10 +3797,10 @@
         <v>1</v>
       </c>
       <c r="G30" s="1" t="s">
-        <v>339</v>
+        <v>341</v>
       </c>
       <c r="H30" s="1" t="s">
-        <v>412</v>
+        <v>420</v>
       </c>
       <c r="I30">
         <f>F30*VALUE(LEFT(H30, FIND(":", H30)-1))</f>
@@ -3757,10 +3829,10 @@
         <v>1</v>
       </c>
       <c r="G31" s="1" t="s">
-        <v>340</v>
+        <v>342</v>
       </c>
       <c r="H31" s="1" t="s">
-        <v>412</v>
+        <v>420</v>
       </c>
       <c r="I31">
         <f>F31*VALUE(LEFT(H31, FIND(":", H31)-1))</f>
@@ -3789,10 +3861,10 @@
         <v>1</v>
       </c>
       <c r="G32" s="1" t="s">
-        <v>341</v>
+        <v>343</v>
       </c>
       <c r="H32" s="1" t="s">
-        <v>412</v>
+        <v>420</v>
       </c>
       <c r="I32">
         <f>F32*VALUE(LEFT(H32, FIND(":", H32)-1))</f>
@@ -3821,10 +3893,10 @@
         <v>1</v>
       </c>
       <c r="G33" s="1" t="s">
-        <v>342</v>
+        <v>344</v>
       </c>
       <c r="H33" s="1" t="s">
-        <v>412</v>
+        <v>420</v>
       </c>
       <c r="I33">
         <f>F33*VALUE(LEFT(H33, FIND(":", H33)-1))</f>
@@ -3855,7 +3927,7 @@
         <v>1</v>
       </c>
       <c r="H34" s="1" t="s">
-        <v>409</v>
+        <v>417</v>
       </c>
       <c r="I34">
         <f>F34*VALUE(LEFT(H34, FIND(":", H34)-1))</f>
@@ -3884,7 +3956,7 @@
         <v>1</v>
       </c>
       <c r="H35" s="1" t="s">
-        <v>409</v>
+        <v>417</v>
       </c>
       <c r="I35">
         <f>F35*VALUE(LEFT(H35, FIND(":", H35)-1))</f>
@@ -3913,7 +3985,7 @@
         <v>1</v>
       </c>
       <c r="H36" s="1" t="s">
-        <v>409</v>
+        <v>417</v>
       </c>
       <c r="I36">
         <f>F36*VALUE(LEFT(H36, FIND(":", H36)-1))</f>
@@ -3942,7 +4014,7 @@
         <v>1</v>
       </c>
       <c r="H37" s="1" t="s">
-        <v>409</v>
+        <v>417</v>
       </c>
       <c r="I37">
         <f>F37*VALUE(LEFT(H37, FIND(":", H37)-1))</f>
@@ -3971,7 +4043,7 @@
         <v>1</v>
       </c>
       <c r="H38" s="1" t="s">
-        <v>409</v>
+        <v>417</v>
       </c>
       <c r="I38">
         <f>F38*VALUE(LEFT(H38, FIND(":", H38)-1))</f>
@@ -4000,7 +4072,7 @@
         <v>1</v>
       </c>
       <c r="H39" s="1" t="s">
-        <v>409</v>
+        <v>417</v>
       </c>
       <c r="I39">
         <f>F39*VALUE(LEFT(H39, FIND(":", H39)-1))</f>
@@ -4031,7 +4103,7 @@
         <v>1</v>
       </c>
       <c r="H40" s="1" t="s">
-        <v>416</v>
+        <v>424</v>
       </c>
       <c r="I40">
         <f>F40*VALUE(LEFT(H40, FIND(":", H40)-1))</f>
@@ -4060,10 +4132,10 @@
         <v>1</v>
       </c>
       <c r="G41" s="1" t="s">
-        <v>343</v>
+        <v>345</v>
       </c>
       <c r="H41" s="1" t="s">
-        <v>412</v>
+        <v>420</v>
       </c>
       <c r="I41">
         <f>F41*VALUE(LEFT(H41, FIND(":", H41)-1))</f>
@@ -4092,10 +4164,10 @@
         <v>1</v>
       </c>
       <c r="G42" s="1" t="s">
-        <v>344</v>
+        <v>346</v>
       </c>
       <c r="H42" s="1" t="s">
-        <v>412</v>
+        <v>420</v>
       </c>
       <c r="I42">
         <f>F42*VALUE(LEFT(H42, FIND(":", H42)-1))</f>
@@ -4124,10 +4196,10 @@
         <v>1</v>
       </c>
       <c r="G43" s="1" t="s">
-        <v>345</v>
+        <v>347</v>
       </c>
       <c r="H43" s="1" t="s">
-        <v>412</v>
+        <v>420</v>
       </c>
       <c r="I43">
         <f>F43*VALUE(LEFT(H43, FIND(":", H43)-1))</f>
@@ -4160,7 +4232,7 @@
         <v>1</v>
       </c>
       <c r="H44" s="1" t="s">
-        <v>417</v>
+        <v>425</v>
       </c>
       <c r="I44">
         <f>F44*VALUE(LEFT(H44, FIND(":", H44)-1))</f>
@@ -4189,10 +4261,10 @@
         <v>1</v>
       </c>
       <c r="G45" s="1" t="s">
-        <v>346</v>
+        <v>348</v>
       </c>
       <c r="H45" s="1" t="s">
-        <v>412</v>
+        <v>420</v>
       </c>
       <c r="I45">
         <f>F45*VALUE(LEFT(H45, FIND(":", H45)-1))</f>
@@ -4221,7 +4293,7 @@
         <v>1</v>
       </c>
       <c r="H46" s="1" t="s">
-        <v>418</v>
+        <v>426</v>
       </c>
       <c r="I46">
         <f>F46*VALUE(LEFT(H46, FIND(":", H46)-1))</f>
@@ -4244,13 +4316,16 @@
         <v>228</v>
       </c>
       <c r="E47" t="s">
-        <v>322</v>
+        <v>326</v>
       </c>
       <c r="F47">
         <v>1</v>
       </c>
+      <c r="G47" s="1" t="s">
+        <v>349</v>
+      </c>
       <c r="H47" s="1" t="s">
-        <v>409</v>
+        <v>420</v>
       </c>
       <c r="I47">
         <f>F47*VALUE(LEFT(H47, FIND(":", H47)-1))</f>
@@ -4273,13 +4348,16 @@
         <v>229</v>
       </c>
       <c r="E48" t="s">
-        <v>322</v>
+        <v>326</v>
       </c>
       <c r="F48">
         <v>1</v>
       </c>
+      <c r="G48" s="1" t="s">
+        <v>350</v>
+      </c>
       <c r="H48" s="1" t="s">
-        <v>409</v>
+        <v>420</v>
       </c>
       <c r="I48">
         <f>F48*VALUE(LEFT(H48, FIND(":", H48)-1))</f>
@@ -4308,7 +4386,7 @@
         <v>1</v>
       </c>
       <c r="H49" s="1" t="s">
-        <v>409</v>
+        <v>417</v>
       </c>
       <c r="I49">
         <f>F49*VALUE(LEFT(H49, FIND(":", H49)-1))</f>
@@ -4337,7 +4415,7 @@
         <v>1</v>
       </c>
       <c r="H50" s="1" t="s">
-        <v>409</v>
+        <v>417</v>
       </c>
       <c r="I50">
         <f>F50*VALUE(LEFT(H50, FIND(":", H50)-1))</f>
@@ -4366,7 +4444,7 @@
         <v>1</v>
       </c>
       <c r="H51" s="1" t="s">
-        <v>409</v>
+        <v>417</v>
       </c>
       <c r="I51">
         <f>F51*VALUE(LEFT(H51, FIND(":", H51)-1))</f>
@@ -4395,10 +4473,10 @@
         <v>1</v>
       </c>
       <c r="G52" s="1" t="s">
-        <v>347</v>
+        <v>351</v>
       </c>
       <c r="H52" s="1" t="s">
-        <v>412</v>
+        <v>420</v>
       </c>
       <c r="I52">
         <f>F52*VALUE(LEFT(H52, FIND(":", H52)-1))</f>
@@ -4427,7 +4505,7 @@
         <v>1</v>
       </c>
       <c r="H53" s="1" t="s">
-        <v>409</v>
+        <v>417</v>
       </c>
       <c r="I53">
         <f>F53*VALUE(LEFT(H53, FIND(":", H53)-1))</f>
@@ -4456,7 +4534,7 @@
         <v>1</v>
       </c>
       <c r="H54" s="1" t="s">
-        <v>409</v>
+        <v>417</v>
       </c>
       <c r="I54">
         <f>F54*VALUE(LEFT(H54, FIND(":", H54)-1))</f>
@@ -4485,7 +4563,7 @@
         <v>1</v>
       </c>
       <c r="H55" s="1" t="s">
-        <v>409</v>
+        <v>417</v>
       </c>
       <c r="I55">
         <f>F55*VALUE(LEFT(H55, FIND(":", H55)-1))</f>
@@ -4516,7 +4594,7 @@
         <v>1</v>
       </c>
       <c r="H56" s="1" t="s">
-        <v>409</v>
+        <v>417</v>
       </c>
       <c r="I56">
         <f>F56*VALUE(LEFT(H56, FIND(":", H56)-1))</f>
@@ -4545,7 +4623,7 @@
         <v>1</v>
       </c>
       <c r="H57" s="1" t="s">
-        <v>409</v>
+        <v>417</v>
       </c>
       <c r="I57">
         <f>F57*VALUE(LEFT(H57, FIND(":", H57)-1))</f>
@@ -4574,7 +4652,7 @@
         <v>1</v>
       </c>
       <c r="H58" s="1" t="s">
-        <v>409</v>
+        <v>417</v>
       </c>
       <c r="I58">
         <f>F58*VALUE(LEFT(H58, FIND(":", H58)-1))</f>
@@ -4603,7 +4681,7 @@
         <v>1</v>
       </c>
       <c r="H59" s="1" t="s">
-        <v>409</v>
+        <v>417</v>
       </c>
       <c r="I59">
         <f>F59*VALUE(LEFT(H59, FIND(":", H59)-1))</f>
@@ -4632,7 +4710,7 @@
         <v>1</v>
       </c>
       <c r="H60" s="1" t="s">
-        <v>409</v>
+        <v>417</v>
       </c>
       <c r="I60">
         <f>F60*VALUE(LEFT(H60, FIND(":", H60)-1))</f>
@@ -4661,7 +4739,7 @@
         <v>1</v>
       </c>
       <c r="H61" s="1" t="s">
-        <v>409</v>
+        <v>417</v>
       </c>
       <c r="I61">
         <f>F61*VALUE(LEFT(H61, FIND(":", H61)-1))</f>
@@ -4692,7 +4770,7 @@
         <v>1</v>
       </c>
       <c r="H62" s="1" t="s">
-        <v>419</v>
+        <v>427</v>
       </c>
       <c r="I62">
         <f>F62*VALUE(LEFT(H62, FIND(":", H62)-1))</f>
@@ -4721,7 +4799,7 @@
         <v>1</v>
       </c>
       <c r="H63" s="1" t="s">
-        <v>409</v>
+        <v>417</v>
       </c>
       <c r="I63">
         <f>F63*VALUE(LEFT(H63, FIND(":", H63)-1))</f>
@@ -4750,7 +4828,7 @@
         <v>1</v>
       </c>
       <c r="H64" s="1" t="s">
-        <v>409</v>
+        <v>417</v>
       </c>
       <c r="I64">
         <f>F64*VALUE(LEFT(H64, FIND(":", H64)-1))</f>
@@ -4779,7 +4857,7 @@
         <v>1</v>
       </c>
       <c r="H65" s="1" t="s">
-        <v>409</v>
+        <v>417</v>
       </c>
       <c r="I65">
         <f>F65*VALUE(LEFT(H65, FIND(":", H65)-1))</f>
@@ -4808,7 +4886,7 @@
         <v>1</v>
       </c>
       <c r="H66" s="1" t="s">
-        <v>409</v>
+        <v>417</v>
       </c>
       <c r="I66">
         <f>F66*VALUE(LEFT(H66, FIND(":", H66)-1))</f>
@@ -4837,7 +4915,7 @@
         <v>1</v>
       </c>
       <c r="H67" s="1" t="s">
-        <v>409</v>
+        <v>417</v>
       </c>
       <c r="I67">
         <f>F67*VALUE(LEFT(H67, FIND(":", H67)-1))</f>
@@ -4868,7 +4946,7 @@
         <v>1</v>
       </c>
       <c r="H68" s="1" t="s">
-        <v>409</v>
+        <v>417</v>
       </c>
       <c r="I68">
         <f>F68*VALUE(LEFT(H68, FIND(":", H68)-1))</f>
@@ -4897,7 +4975,7 @@
         <v>1</v>
       </c>
       <c r="H69" s="1" t="s">
-        <v>409</v>
+        <v>417</v>
       </c>
       <c r="I69">
         <f>F69*VALUE(LEFT(H69, FIND(":", H69)-1))</f>
@@ -4926,7 +5004,7 @@
         <v>1</v>
       </c>
       <c r="H70" s="1" t="s">
-        <v>409</v>
+        <v>417</v>
       </c>
       <c r="I70">
         <f>F70*VALUE(LEFT(H70, FIND(":", H70)-1))</f>
@@ -4955,7 +5033,7 @@
         <v>1</v>
       </c>
       <c r="H71" s="1" t="s">
-        <v>409</v>
+        <v>417</v>
       </c>
       <c r="I71">
         <f>F71*VALUE(LEFT(H71, FIND(":", H71)-1))</f>
@@ -4984,7 +5062,7 @@
         <v>1</v>
       </c>
       <c r="H72" s="1" t="s">
-        <v>409</v>
+        <v>417</v>
       </c>
       <c r="I72">
         <f>F72*VALUE(LEFT(H72, FIND(":", H72)-1))</f>
@@ -5013,10 +5091,10 @@
         <v>1</v>
       </c>
       <c r="G73" s="1" t="s">
-        <v>348</v>
+        <v>352</v>
       </c>
       <c r="H73" s="1" t="s">
-        <v>412</v>
+        <v>420</v>
       </c>
       <c r="I73">
         <f>F73*VALUE(LEFT(H73, FIND(":", H73)-1))</f>
@@ -5047,7 +5125,7 @@
         <v>1</v>
       </c>
       <c r="H74" s="1" t="s">
-        <v>409</v>
+        <v>417</v>
       </c>
       <c r="I74">
         <f>F74*VALUE(LEFT(H74, FIND(":", H74)-1))</f>
@@ -5076,7 +5154,7 @@
         <v>1</v>
       </c>
       <c r="H75" s="1" t="s">
-        <v>420</v>
+        <v>428</v>
       </c>
       <c r="I75">
         <f>F75*VALUE(LEFT(H75, FIND(":", H75)-1))</f>
@@ -5105,7 +5183,7 @@
         <v>1</v>
       </c>
       <c r="H76" s="1" t="s">
-        <v>419</v>
+        <v>427</v>
       </c>
       <c r="I76">
         <f>F76*VALUE(LEFT(H76, FIND(":", H76)-1))</f>
@@ -5134,7 +5212,7 @@
         <v>1</v>
       </c>
       <c r="H77" s="1" t="s">
-        <v>409</v>
+        <v>417</v>
       </c>
       <c r="I77">
         <f>F77*VALUE(LEFT(H77, FIND(":", H77)-1))</f>
@@ -5163,7 +5241,7 @@
         <v>1</v>
       </c>
       <c r="H78" s="1" t="s">
-        <v>409</v>
+        <v>417</v>
       </c>
       <c r="I78">
         <f>F78*VALUE(LEFT(H78, FIND(":", H78)-1))</f>
@@ -5192,7 +5270,7 @@
         <v>1</v>
       </c>
       <c r="H79" s="1" t="s">
-        <v>409</v>
+        <v>417</v>
       </c>
       <c r="I79">
         <f>F79*VALUE(LEFT(H79, FIND(":", H79)-1))</f>
@@ -5225,7 +5303,7 @@
         <v>1</v>
       </c>
       <c r="H80" s="1" t="s">
-        <v>409</v>
+        <v>417</v>
       </c>
       <c r="I80">
         <f>F80*VALUE(LEFT(H80, FIND(":", H80)-1))</f>
@@ -5254,7 +5332,7 @@
         <v>1</v>
       </c>
       <c r="H81" s="1" t="s">
-        <v>409</v>
+        <v>417</v>
       </c>
       <c r="I81">
         <f>F81*VALUE(LEFT(H81, FIND(":", H81)-1))</f>
@@ -5283,7 +5361,7 @@
         <v>1</v>
       </c>
       <c r="H82" s="1" t="s">
-        <v>409</v>
+        <v>417</v>
       </c>
       <c r="I82">
         <f>F82*VALUE(LEFT(H82, FIND(":", H82)-1))</f>
@@ -5312,7 +5390,7 @@
         <v>1</v>
       </c>
       <c r="H83" s="1" t="s">
-        <v>409</v>
+        <v>417</v>
       </c>
       <c r="I83">
         <f>F83*VALUE(LEFT(H83, FIND(":", H83)-1))</f>
@@ -5341,7 +5419,7 @@
         <v>1</v>
       </c>
       <c r="H84" s="1" t="s">
-        <v>421</v>
+        <v>429</v>
       </c>
       <c r="I84">
         <f>F84*VALUE(LEFT(H84, FIND(":", H84)-1))</f>
@@ -5370,7 +5448,7 @@
         <v>1</v>
       </c>
       <c r="H85" s="1" t="s">
-        <v>409</v>
+        <v>417</v>
       </c>
       <c r="I85">
         <f>F85*VALUE(LEFT(H85, FIND(":", H85)-1))</f>
@@ -5401,7 +5479,7 @@
         <v>1</v>
       </c>
       <c r="H86" s="1" t="s">
-        <v>417</v>
+        <v>425</v>
       </c>
       <c r="I86">
         <f>F86*VALUE(LEFT(H86, FIND(":", H86)-1))</f>
@@ -5430,7 +5508,7 @@
         <v>1</v>
       </c>
       <c r="H87" s="1" t="s">
-        <v>417</v>
+        <v>425</v>
       </c>
       <c r="I87">
         <f>F87*VALUE(LEFT(H87, FIND(":", H87)-1))</f>
@@ -5459,7 +5537,7 @@
         <v>1</v>
       </c>
       <c r="H88" s="1" t="s">
-        <v>409</v>
+        <v>417</v>
       </c>
       <c r="I88">
         <f>F88*VALUE(LEFT(H88, FIND(":", H88)-1))</f>
@@ -5488,7 +5566,7 @@
         <v>1</v>
       </c>
       <c r="H89" s="1" t="s">
-        <v>409</v>
+        <v>417</v>
       </c>
       <c r="I89">
         <f>F89*VALUE(LEFT(H89, FIND(":", H89)-1))</f>
@@ -5517,7 +5595,7 @@
         <v>1</v>
       </c>
       <c r="H90" s="1" t="s">
-        <v>409</v>
+        <v>417</v>
       </c>
       <c r="I90">
         <f>F90*VALUE(LEFT(H90, FIND(":", H90)-1))</f>
@@ -5546,7 +5624,7 @@
         <v>1</v>
       </c>
       <c r="H91" s="1" t="s">
-        <v>409</v>
+        <v>417</v>
       </c>
       <c r="I91">
         <f>F91*VALUE(LEFT(H91, FIND(":", H91)-1))</f>
@@ -5577,7 +5655,7 @@
         <v>1</v>
       </c>
       <c r="H92" s="1" t="s">
-        <v>409</v>
+        <v>417</v>
       </c>
       <c r="I92">
         <f>F92*VALUE(LEFT(H92, FIND(":", H92)-1))</f>
@@ -5600,16 +5678,16 @@
         <v>274</v>
       </c>
       <c r="E93" t="s">
-        <v>323</v>
+        <v>327</v>
       </c>
       <c r="F93">
         <v>1</v>
       </c>
       <c r="G93" s="1" t="s">
-        <v>349</v>
+        <v>353</v>
       </c>
       <c r="H93" s="1" t="s">
-        <v>412</v>
+        <v>420</v>
       </c>
       <c r="I93">
         <f>F93*VALUE(LEFT(H93, FIND(":", H93)-1))</f>
@@ -5632,13 +5710,13 @@
         <v>275</v>
       </c>
       <c r="E94" t="s">
-        <v>323</v>
+        <v>327</v>
       </c>
       <c r="F94">
         <v>1</v>
       </c>
       <c r="H94" s="1" t="s">
-        <v>422</v>
+        <v>430</v>
       </c>
       <c r="I94">
         <f>F94*VALUE(LEFT(H94, FIND(":", H94)-1))</f>
@@ -5667,10 +5745,10 @@
         <v>1</v>
       </c>
       <c r="G95" s="1" t="s">
-        <v>350</v>
+        <v>354</v>
       </c>
       <c r="H95" s="1" t="s">
-        <v>419</v>
+        <v>427</v>
       </c>
       <c r="I95">
         <f>F95*VALUE(LEFT(H95, FIND(":", H95)-1))</f>
@@ -5699,7 +5777,7 @@
         <v>1</v>
       </c>
       <c r="H96" s="1" t="s">
-        <v>423</v>
+        <v>431</v>
       </c>
       <c r="I96">
         <f>F96*VALUE(LEFT(H96, FIND(":", H96)-1))</f>
@@ -5728,10 +5806,10 @@
         <v>1</v>
       </c>
       <c r="G97" s="1" t="s">
-        <v>351</v>
+        <v>355</v>
       </c>
       <c r="H97" s="1" t="s">
-        <v>412</v>
+        <v>420</v>
       </c>
       <c r="I97">
         <f>F97*VALUE(LEFT(H97, FIND(":", H97)-1))</f>
@@ -5762,10 +5840,10 @@
         <v>1</v>
       </c>
       <c r="G98" s="1" t="s">
-        <v>352</v>
+        <v>356</v>
       </c>
       <c r="H98" s="1" t="s">
-        <v>412</v>
+        <v>420</v>
       </c>
       <c r="I98">
         <f>F98*VALUE(LEFT(H98, FIND(":", H98)-1))</f>
@@ -5794,10 +5872,10 @@
         <v>1</v>
       </c>
       <c r="G99" s="1" t="s">
-        <v>353</v>
+        <v>357</v>
       </c>
       <c r="H99" s="1" t="s">
-        <v>412</v>
+        <v>420</v>
       </c>
       <c r="I99">
         <f>F99*VALUE(LEFT(H99, FIND(":", H99)-1))</f>
@@ -5826,10 +5904,10 @@
         <v>1</v>
       </c>
       <c r="G100" s="1" t="s">
-        <v>354</v>
+        <v>358</v>
       </c>
       <c r="H100" s="1" t="s">
-        <v>412</v>
+        <v>420</v>
       </c>
       <c r="I100">
         <f>F100*VALUE(LEFT(H100, FIND(":", H100)-1))</f>
@@ -5858,10 +5936,10 @@
         <v>1</v>
       </c>
       <c r="G101" s="1" t="s">
-        <v>355</v>
+        <v>359</v>
       </c>
       <c r="H101" s="1" t="s">
-        <v>412</v>
+        <v>420</v>
       </c>
       <c r="I101">
         <f>F101*VALUE(LEFT(H101, FIND(":", H101)-1))</f>
@@ -5890,10 +5968,10 @@
         <v>1</v>
       </c>
       <c r="G102" s="1" t="s">
-        <v>356</v>
+        <v>360</v>
       </c>
       <c r="H102" s="1" t="s">
-        <v>412</v>
+        <v>420</v>
       </c>
       <c r="I102">
         <f>F102*VALUE(LEFT(H102, FIND(":", H102)-1))</f>
@@ -5922,7 +6000,7 @@
         <v>1</v>
       </c>
       <c r="H103" s="1" t="s">
-        <v>419</v>
+        <v>427</v>
       </c>
       <c r="I103">
         <f>F103*VALUE(LEFT(H103, FIND(":", H103)-1))</f>
@@ -5951,10 +6029,10 @@
         <v>1</v>
       </c>
       <c r="G104" s="1" t="s">
-        <v>357</v>
+        <v>361</v>
       </c>
       <c r="H104" s="1" t="s">
-        <v>412</v>
+        <v>420</v>
       </c>
       <c r="I104">
         <f>F104*VALUE(LEFT(H104, FIND(":", H104)-1))</f>
@@ -5985,10 +6063,10 @@
         <v>1</v>
       </c>
       <c r="G105" s="1" t="s">
-        <v>358</v>
+        <v>362</v>
       </c>
       <c r="H105" s="1" t="s">
-        <v>412</v>
+        <v>420</v>
       </c>
       <c r="I105">
         <f>F105*VALUE(LEFT(H105, FIND(":", H105)-1))</f>
@@ -6017,10 +6095,10 @@
         <v>1</v>
       </c>
       <c r="G106" s="1" t="s">
-        <v>359</v>
+        <v>363</v>
       </c>
       <c r="H106" s="1" t="s">
-        <v>412</v>
+        <v>420</v>
       </c>
       <c r="I106">
         <f>F106*VALUE(LEFT(H106, FIND(":", H106)-1))</f>
@@ -6049,10 +6127,10 @@
         <v>1</v>
       </c>
       <c r="G107" s="1" t="s">
-        <v>360</v>
+        <v>364</v>
       </c>
       <c r="H107" s="1" t="s">
-        <v>412</v>
+        <v>420</v>
       </c>
       <c r="I107">
         <f>F107*VALUE(LEFT(H107, FIND(":", H107)-1))</f>
@@ -6081,10 +6159,10 @@
         <v>1</v>
       </c>
       <c r="G108" s="1" t="s">
-        <v>361</v>
+        <v>365</v>
       </c>
       <c r="H108" s="1" t="s">
-        <v>412</v>
+        <v>420</v>
       </c>
       <c r="I108">
         <f>F108*VALUE(LEFT(H108, FIND(":", H108)-1))</f>
@@ -6113,10 +6191,10 @@
         <v>1</v>
       </c>
       <c r="G109" s="1" t="s">
-        <v>362</v>
+        <v>366</v>
       </c>
       <c r="H109" s="1" t="s">
-        <v>412</v>
+        <v>420</v>
       </c>
       <c r="I109">
         <f>F109*VALUE(LEFT(H109, FIND(":", H109)-1))</f>
@@ -6145,7 +6223,7 @@
         <v>1</v>
       </c>
       <c r="H110" s="1" t="s">
-        <v>422</v>
+        <v>430</v>
       </c>
       <c r="I110">
         <f>F110*VALUE(LEFT(H110, FIND(":", H110)-1))</f>
@@ -6178,10 +6256,10 @@
         <v>1</v>
       </c>
       <c r="G111" s="1" t="s">
-        <v>363</v>
+        <v>367</v>
       </c>
       <c r="H111" s="1" t="s">
-        <v>412</v>
+        <v>420</v>
       </c>
       <c r="I111">
         <f>F111*VALUE(LEFT(H111, FIND(":", H111)-1))</f>
@@ -6210,10 +6288,10 @@
         <v>1</v>
       </c>
       <c r="G112" s="1" t="s">
-        <v>364</v>
+        <v>368</v>
       </c>
       <c r="H112" s="1" t="s">
-        <v>419</v>
+        <v>427</v>
       </c>
       <c r="I112">
         <f>F112*VALUE(LEFT(H112, FIND(":", H112)-1))</f>
@@ -6242,10 +6320,10 @@
         <v>1</v>
       </c>
       <c r="G113" s="1" t="s">
-        <v>365</v>
+        <v>369</v>
       </c>
       <c r="H113" s="1" t="s">
-        <v>412</v>
+        <v>420</v>
       </c>
       <c r="I113">
         <f>F113*VALUE(LEFT(H113, FIND(":", H113)-1))</f>
@@ -6274,10 +6352,10 @@
         <v>1</v>
       </c>
       <c r="G114" s="1" t="s">
-        <v>366</v>
+        <v>370</v>
       </c>
       <c r="H114" s="1" t="s">
-        <v>419</v>
+        <v>427</v>
       </c>
       <c r="I114">
         <f>F114*VALUE(LEFT(H114, FIND(":", H114)-1))</f>
@@ -6306,10 +6384,10 @@
         <v>1</v>
       </c>
       <c r="G115" s="1" t="s">
-        <v>367</v>
+        <v>371</v>
       </c>
       <c r="H115" s="1" t="s">
-        <v>419</v>
+        <v>427</v>
       </c>
       <c r="I115">
         <f>F115*VALUE(LEFT(H115, FIND(":", H115)-1))</f>
@@ -6338,10 +6416,10 @@
         <v>1</v>
       </c>
       <c r="G116" s="1" t="s">
-        <v>368</v>
+        <v>372</v>
       </c>
       <c r="H116" s="1" t="s">
-        <v>412</v>
+        <v>420</v>
       </c>
       <c r="I116">
         <f>F116*VALUE(LEFT(H116, FIND(":", H116)-1))</f>
@@ -6370,7 +6448,7 @@
         <v>1</v>
       </c>
       <c r="H117" s="1" t="s">
-        <v>409</v>
+        <v>417</v>
       </c>
       <c r="I117">
         <f>F117*VALUE(LEFT(H117, FIND(":", H117)-1))</f>
@@ -6401,10 +6479,10 @@
         <v>1</v>
       </c>
       <c r="G118" s="1" t="s">
-        <v>369</v>
+        <v>373</v>
       </c>
       <c r="H118" s="1" t="s">
-        <v>412</v>
+        <v>420</v>
       </c>
       <c r="I118">
         <f>F118*VALUE(LEFT(H118, FIND(":", H118)-1))</f>
@@ -6433,10 +6511,10 @@
         <v>1</v>
       </c>
       <c r="G119" s="1" t="s">
-        <v>370</v>
+        <v>374</v>
       </c>
       <c r="H119" s="1" t="s">
-        <v>412</v>
+        <v>420</v>
       </c>
       <c r="I119">
         <f>F119*VALUE(LEFT(H119, FIND(":", H119)-1))</f>
@@ -6465,7 +6543,7 @@
         <v>1</v>
       </c>
       <c r="H120" s="1" t="s">
-        <v>424</v>
+        <v>432</v>
       </c>
       <c r="I120">
         <f>F120*VALUE(LEFT(H120, FIND(":", H120)-1))</f>
@@ -6493,8 +6571,11 @@
       <c r="F121">
         <v>1</v>
       </c>
+      <c r="G121" s="1" t="s">
+        <v>375</v>
+      </c>
       <c r="H121" s="1" t="s">
-        <v>409</v>
+        <v>420</v>
       </c>
       <c r="I121">
         <f>F121*VALUE(LEFT(H121, FIND(":", H121)-1))</f>
@@ -6522,8 +6603,11 @@
       <c r="F122">
         <v>1</v>
       </c>
+      <c r="G122" s="1" t="s">
+        <v>376</v>
+      </c>
       <c r="H122" s="1" t="s">
-        <v>409</v>
+        <v>420</v>
       </c>
       <c r="I122">
         <f>F122*VALUE(LEFT(H122, FIND(":", H122)-1))</f>
@@ -6552,10 +6636,10 @@
         <v>1</v>
       </c>
       <c r="G123" s="1" t="s">
-        <v>371</v>
+        <v>377</v>
       </c>
       <c r="H123" s="1" t="s">
-        <v>412</v>
+        <v>420</v>
       </c>
       <c r="I123">
         <f>F123*VALUE(LEFT(H123, FIND(":", H123)-1))</f>
@@ -6583,8 +6667,11 @@
       <c r="F124">
         <v>1</v>
       </c>
+      <c r="G124" s="1" t="s">
+        <v>378</v>
+      </c>
       <c r="H124" s="1" t="s">
-        <v>409</v>
+        <v>433</v>
       </c>
       <c r="I124">
         <f>F124*VALUE(LEFT(H124, FIND(":", H124)-1))</f>
@@ -6615,7 +6702,7 @@
         <v>1</v>
       </c>
       <c r="H125" s="1" t="s">
-        <v>409</v>
+        <v>417</v>
       </c>
       <c r="I125">
         <f>F125*VALUE(LEFT(H125, FIND(":", H125)-1))</f>
@@ -6644,7 +6731,7 @@
         <v>1</v>
       </c>
       <c r="H126" s="1" t="s">
-        <v>409</v>
+        <v>417</v>
       </c>
       <c r="I126">
         <f>F126*VALUE(LEFT(H126, FIND(":", H126)-1))</f>
@@ -6673,7 +6760,7 @@
         <v>1</v>
       </c>
       <c r="H127" s="1" t="s">
-        <v>409</v>
+        <v>417</v>
       </c>
       <c r="I127">
         <f>F127*VALUE(LEFT(H127, FIND(":", H127)-1))</f>
@@ -6702,7 +6789,7 @@
         <v>1</v>
       </c>
       <c r="H128" s="1" t="s">
-        <v>425</v>
+        <v>434</v>
       </c>
       <c r="I128">
         <f>F128*VALUE(LEFT(H128, FIND(":", H128)-1))</f>
@@ -6731,7 +6818,7 @@
         <v>1</v>
       </c>
       <c r="H129" s="1" t="s">
-        <v>409</v>
+        <v>417</v>
       </c>
       <c r="I129">
         <f>F129*VALUE(LEFT(H129, FIND(":", H129)-1))</f>
@@ -6760,10 +6847,10 @@
         <v>1</v>
       </c>
       <c r="G130" s="1" t="s">
-        <v>372</v>
+        <v>379</v>
       </c>
       <c r="H130" s="1" t="s">
-        <v>412</v>
+        <v>420</v>
       </c>
       <c r="I130">
         <f>F130*VALUE(LEFT(H130, FIND(":", H130)-1))</f>
@@ -6792,10 +6879,10 @@
         <v>1</v>
       </c>
       <c r="G131" s="1" t="s">
-        <v>373</v>
+        <v>380</v>
       </c>
       <c r="H131" s="1" t="s">
-        <v>412</v>
+        <v>420</v>
       </c>
       <c r="I131">
         <f>F131*VALUE(LEFT(H131, FIND(":", H131)-1))</f>
@@ -6824,7 +6911,7 @@
         <v>1</v>
       </c>
       <c r="H132" s="1" t="s">
-        <v>409</v>
+        <v>417</v>
       </c>
       <c r="I132">
         <f>F132*VALUE(LEFT(H132, FIND(":", H132)-1))</f>
@@ -6847,13 +6934,13 @@
         <v>314</v>
       </c>
       <c r="E133" t="s">
-        <v>326</v>
+        <v>328</v>
       </c>
       <c r="F133">
         <v>1</v>
       </c>
       <c r="H133" s="1" t="s">
-        <v>425</v>
+        <v>434</v>
       </c>
       <c r="I133">
         <f>F133*VALUE(LEFT(H133, FIND(":", H133)-1))</f>
@@ -6884,7 +6971,7 @@
         <v>1</v>
       </c>
       <c r="H134" s="1" t="s">
-        <v>409</v>
+        <v>417</v>
       </c>
       <c r="I134">
         <f>F134*VALUE(LEFT(H134, FIND(":", H134)-1))</f>
@@ -6913,10 +7000,10 @@
         <v>1</v>
       </c>
       <c r="G135" s="1" t="s">
-        <v>374</v>
+        <v>381</v>
       </c>
       <c r="H135" s="1" t="s">
-        <v>412</v>
+        <v>420</v>
       </c>
       <c r="I135">
         <f>F135*VALUE(LEFT(H135, FIND(":", H135)-1))</f>
@@ -6945,10 +7032,10 @@
         <v>1</v>
       </c>
       <c r="G136" s="1" t="s">
-        <v>375</v>
+        <v>382</v>
       </c>
       <c r="H136" s="1" t="s">
-        <v>412</v>
+        <v>420</v>
       </c>
       <c r="I136">
         <f>F136*VALUE(LEFT(H136, FIND(":", H136)-1))</f>
@@ -6977,7 +7064,7 @@
         <v>1</v>
       </c>
       <c r="H137" s="1" t="s">
-        <v>409</v>
+        <v>417</v>
       </c>
       <c r="I137">
         <f>F137*VALUE(LEFT(H137, FIND(":", H137)-1))</f>
@@ -7006,7 +7093,7 @@
         <v>1</v>
       </c>
       <c r="H138" s="1" t="s">
-        <v>426</v>
+        <v>435</v>
       </c>
       <c r="I138">
         <f>F138*VALUE(LEFT(H138, FIND(":", H138)-1))</f>
@@ -7035,7 +7122,7 @@
         <v>1</v>
       </c>
       <c r="H139" s="1" t="s">
-        <v>409</v>
+        <v>417</v>
       </c>
       <c r="I139">
         <f>F139*VALUE(LEFT(H139, FIND(":", H139)-1))</f>
@@ -7064,7 +7151,7 @@
         <v>1</v>
       </c>
       <c r="H140" s="1" t="s">
-        <v>409</v>
+        <v>417</v>
       </c>
       <c r="I140">
         <f>F140*VALUE(LEFT(H140, FIND(":", H140)-1))</f>
@@ -7243,10 +7330,10 @@
       <formula1>"0: No documented method,10: Documented method of assessing modernization efforts"</formula1>
     </dataValidation>
     <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="H47">
-      <formula1>"0: Not done,10: Completed"</formula1>
+      <formula1>"0: No items completed,2: 1 item completed,4: 2 items completed,6: 3 items completed,8: 4 items completed,10: 5 items completed"</formula1>
     </dataValidation>
     <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="H48">
-      <formula1>"0: Not done,10: Completed"</formula1>
+      <formula1>"0: No items completed,3: 1 item completed,5: 2 items completed,8: 3 items completed,10: 4 items completed"</formula1>
     </dataValidation>
     <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="H49">
       <formula1>"0: Not done,10: Completed"</formula1>
@@ -7465,16 +7552,16 @@
       <formula1>"0: No alerting to any owners,1: Alerting in at least one owner,3: Alerting to some owners [&gt;20%],6: Alerting to most owners [&gt;60%],10: Alerting to all owners [100%]"</formula1>
     </dataValidation>
     <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="H121">
-      <formula1>"0: Not done,10: Completed"</formula1>
+      <formula1>"0: No items completed,2: 1 item completed,4: 2 items completed,5: 3 items completed,7: 4 items completed,9: 5 items completed,10: 6 items completed"</formula1>
     </dataValidation>
     <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="H122">
-      <formula1>"0: Not done,10: Completed"</formula1>
+      <formula1>"0: No items completed,2: item 1 completed,4: items 1-2 completed,6: items 1-3 completed,8: items 1-4 completed,10: items 1-5 completed"</formula1>
     </dataValidation>
     <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="H123">
       <formula1>"0: No items completed,2: 1 item completed,3: 2 items completed,4: 3 items completed,5: 4 items completed,7: 5 items completed,8: 6 items completed,9: 7 items completed,10: 8 items completed"</formula1>
     </dataValidation>
     <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="H124">
-      <formula1>"0: Not done,10: Completed"</formula1>
+      <formula1>"0: Low Maturity. Score Range (0-14),4: Developing. Score Range (15-30),7: Established. Score Range (31-42),10: Optimizing. Score Range (43-50)"</formula1>
     </dataValidation>
     <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="H125">
       <formula1>"0: Not done,10: Completed"</formula1>

</xml_diff>